<commit_message>
Sincronização automática: 05/05/2026  8:24:19.33
</commit_message>
<xml_diff>
--- a/dados/OS_192/Fazenda_OS192_amostras_simples.xlsx
+++ b/dados/OS_192/Fazenda_OS192_amostras_simples.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Agroserver\gestao_projetos\08_Processo_Químico\02_Clientes\_teste_dash_custos_quimico\OS_192\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C90BF8D-BB5A-43E9-94D6-4531223FE8EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1457CCF3-3041-4E64-8425-6DFAC4E7C40A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1102,9 +1102,6 @@
     <t>ASP25005601920467A11S250061</t>
   </si>
   <si>
-    <t>CNH</t>
-  </si>
-  <si>
     <t>P_Resina</t>
   </si>
   <si>
@@ -1121,6 +1118,9 @@
   </si>
   <si>
     <t>pH_H2O</t>
+  </si>
+  <si>
+    <t>CHN</t>
   </si>
 </sst>
 </file>
@@ -1591,13 +1591,13 @@
         <v>13</v>
       </c>
       <c r="P1" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="Q1" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>360</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>361</v>
       </c>
       <c r="S1" s="3" t="s">
         <v>40</v>
@@ -1606,13 +1606,13 @@
         <v>41</v>
       </c>
       <c r="U1" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="V1" s="3" t="s">
         <v>362</v>
       </c>
-      <c r="V1" s="3" t="s">
-        <v>363</v>
-      </c>
       <c r="W1" s="3" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="X1" s="3" t="s">
         <v>42</v>
@@ -1621,7 +1621,7 @@
         <v>43</v>
       </c>
       <c r="Z1" s="3" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="AA1" s="1" t="s">
         <v>14</v>

</xml_diff>